<commit_message>
Update FRS crosswalk brief and AFS table outputs
- Update FRS crosswalk brief with latest findings
- Regenerate AFS table outputs (air program, facilities, historical compliance)
- Minor updates to table generation scripts

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/tables/afs_air_program_table.xlsx
+++ b/output/tables/afs_air_program_table.xlsx
@@ -104,7 +104,7 @@
     <t xml:space="preserve">SM - Synthetic minor: below all major thresholds via enforceable limits</t>
   </si>
   <si>
-    <t xml:space="preserve">C - Unknown</t>
+    <t xml:space="preserve">C - Unregulated pollutant: actual/potential controlled emissions &gt;100 tons/year</t>
   </si>
   <si>
     <t xml:space="preserve">ND - Thresholds not defined</t>
@@ -123,7 +123,7 @@
 EPA compliance status code for the facility under this program.</t>
   </si>
   <si>
-    <t xml:space="preserve">C</t>
+    <t xml:space="preserve">C - In Compliance With Procedural Requirements</t>
   </si>
   <si>
     <t xml:space="preserve">4 - In Compliance, Certification</t>

</xml_diff>